<commit_message>
Weekly TRQ update 2026-09-21
</commit_message>
<xml_diff>
--- a/data/canada_trq_tracker.xlsx
+++ b/data/canada_trq_tracker.xlsx
@@ -12390,7 +12390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12481,7 +12481,12 @@
           <t>September 14 2026</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>September 21 2026</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -12540,6 +12545,9 @@
       <c r="Q3" s="4" t="n">
         <v>0.3369</v>
       </c>
+      <c r="R3" s="4" t="n">
+        <v>0.3369</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12591,6 +12599,9 @@
       <c r="Q4" s="4" t="n">
         <v>0.0396</v>
       </c>
+      <c r="R4" s="4" t="n">
+        <v>0.0436</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12636,6 +12647,9 @@
       <c r="Q5" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="R5" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12700,6 +12714,10 @@
         <f>SUM(Q3:Q5)</f>
         <v/>
       </c>
+      <c r="R6" s="5">
+        <f>SUM(R3:R5)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12754,6 +12772,9 @@
       <c r="Q7" s="4" t="n">
         <v>0.3542</v>
       </c>
+      <c r="R7" s="4" t="n">
+        <v>0.3542</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12802,6 +12823,9 @@
       <c r="Q8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12829,6 +12853,9 @@
       <c r="Q9" s="4" t="n">
         <v>0.3547</v>
       </c>
+      <c r="R9" s="4" t="n">
+        <v>0.3547</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12871,6 +12898,9 @@
       <c r="Q11" s="4" t="n">
         <v>0.1897</v>
       </c>
+      <c r="R11" s="4" t="n">
+        <v>0.2734</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12935,6 +12965,10 @@
         <f>SUM(Q7:Q11)</f>
         <v/>
       </c>
+      <c r="R12" s="5">
+        <f>SUM(R7:R11)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12989,6 +13023,9 @@
       <c r="Q13" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="R13" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13043,6 +13080,9 @@
       <c r="Q14" s="4" t="n">
         <v>0.1135</v>
       </c>
+      <c r="R14" s="4" t="n">
+        <v>0.1135</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13097,6 +13137,9 @@
       <c r="Q15" s="4" t="n">
         <v>0.5222</v>
       </c>
+      <c r="R15" s="4" t="n">
+        <v>0.5222</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13148,6 +13191,9 @@
       <c r="Q16" s="4" t="n">
         <v>0.0008</v>
       </c>
+      <c r="R16" s="4" t="n">
+        <v>0.0008</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13199,6 +13245,9 @@
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R17" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13250,6 +13299,9 @@
       <c r="Q18" s="4" t="n">
         <v>0.3156</v>
       </c>
+      <c r="R18" s="4" t="n">
+        <v>0.3156</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13298,6 +13350,9 @@
       <c r="Q19" s="4" t="n">
         <v>0.0406</v>
       </c>
+      <c r="R19" s="4" t="n">
+        <v>0.0406</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13346,6 +13401,9 @@
       <c r="Q20" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R20" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13410,6 +13468,10 @@
         <f>SUM(Q13:Q20)</f>
         <v/>
       </c>
+      <c r="R21" s="5">
+        <f>SUM(R13:R20)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13464,6 +13526,9 @@
       <c r="Q22" s="4" t="n">
         <v>0.003</v>
       </c>
+      <c r="R22" s="4" t="n">
+        <v>0.003</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13518,6 +13583,9 @@
       <c r="Q23" s="4" t="n">
         <v>0.2673</v>
       </c>
+      <c r="R23" s="4" t="n">
+        <v>0.2673</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13572,6 +13640,9 @@
       <c r="Q24" s="4" t="n">
         <v>0.0069</v>
       </c>
+      <c r="R24" s="4" t="n">
+        <v>0.0069</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13626,6 +13697,9 @@
       <c r="Q25" s="4" t="n">
         <v>0.2488</v>
       </c>
+      <c r="R25" s="4" t="n">
+        <v>0.2488</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13680,6 +13754,9 @@
       <c r="Q26" s="4" t="n">
         <v>0.3697</v>
       </c>
+      <c r="R26" s="4" t="n">
+        <v>0.3697</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13734,6 +13811,9 @@
       <c r="Q27" s="4" t="n">
         <v>0.0289</v>
       </c>
+      <c r="R27" s="4" t="n">
+        <v>0.0289</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13785,6 +13865,9 @@
       <c r="Q28" s="4" t="n">
         <v>0.07539999999999999</v>
       </c>
+      <c r="R28" s="4" t="n">
+        <v>0.07539999999999999</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13849,6 +13932,10 @@
         <f>SUM(Q22:Q28)</f>
         <v/>
       </c>
+      <c r="R29" s="5">
+        <f>SUM(R22:R28)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13903,7 +13990,10 @@
       <c r="Q30" s="4" t="n">
         <v>0.29</v>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="R30" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="S30" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -13962,6 +14052,9 @@
       <c r="Q31" s="4" t="n">
         <v>0.0037</v>
       </c>
+      <c r="R31" s="4" t="n">
+        <v>0.0037</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14016,6 +14109,9 @@
       <c r="Q32" s="4" t="n">
         <v>0.2899</v>
       </c>
+      <c r="R32" s="4" t="n">
+        <v>0.2899</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14070,6 +14166,9 @@
       <c r="Q33" s="4" t="n">
         <v>0.0883</v>
       </c>
+      <c r="R33" s="4" t="n">
+        <v>0.0883</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14115,6 +14214,9 @@
       <c r="Q34" s="4" t="n">
         <v>0.0113</v>
       </c>
+      <c r="R34" s="4" t="n">
+        <v>0.0113</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14139,6 +14241,9 @@
       <c r="Q35" s="4" t="n">
         <v>0.2822</v>
       </c>
+      <c r="R35" s="4" t="n">
+        <v>0.2822</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14203,6 +14308,10 @@
         <f>SUM(Q30:Q35)</f>
         <v/>
       </c>
+      <c r="R36" s="5">
+        <f>SUM(R30:R35)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14257,6 +14366,9 @@
       <c r="Q37" s="4" t="n">
         <v>0.1576</v>
       </c>
+      <c r="R37" s="4" t="n">
+        <v>0.1576</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14311,7 +14423,10 @@
       <c r="Q38" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="R38" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="S38" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14370,7 +14485,10 @@
       <c r="Q39" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="R39" s="4" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="S39" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14426,6 +14544,9 @@
       <c r="Q40" s="4" t="n">
         <v>0.0024</v>
       </c>
+      <c r="R40" s="4" t="n">
+        <v>0.0024</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14490,6 +14611,10 @@
         <f>SUM(Q37:Q40)</f>
         <v/>
       </c>
+      <c r="R41" s="5">
+        <f>SUM(R37:R40)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14532,6 +14657,14 @@
       <c r="Q42" s="4" t="n">
         <v>0.4069</v>
       </c>
+      <c r="R42" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14571,7 +14704,10 @@
       <c r="Q43" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="R43" t="inlineStr">
+      <c r="R43" s="4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="S43" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -14640,6 +14776,10 @@
         <f>SUM(Q42:Q43)</f>
         <v/>
       </c>
+      <c r="R44" s="5">
+        <f>SUM(R42:R43)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14694,6 +14834,9 @@
       <c r="Q45" s="4" t="n">
         <v>0.0146</v>
       </c>
+      <c r="R45" s="4" t="n">
+        <v>0.0146</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14748,6 +14891,9 @@
       <c r="Q46" s="4" t="n">
         <v>0.2065</v>
       </c>
+      <c r="R46" s="4" t="n">
+        <v>0.2065</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14802,6 +14948,9 @@
       <c r="Q47" s="4" t="n">
         <v>0.3483</v>
       </c>
+      <c r="R47" s="4" t="n">
+        <v>0.3483</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14856,6 +15005,9 @@
       <c r="Q48" s="4" t="n">
         <v>0.4306</v>
       </c>
+      <c r="R48" s="4" t="n">
+        <v>0.4306</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -14918,6 +15070,10 @@
       </c>
       <c r="Q49" s="5">
         <f>SUM(Q45:Q48)</f>
+        <v/>
+      </c>
+      <c r="R49" s="5">
+        <f>SUM(R45:R48)</f>
         <v/>
       </c>
     </row>
@@ -14932,7 +15088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:S80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15023,7 +15179,12 @@
           <t>September 14 2026</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>September 21 2026</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>OVER</t>
         </is>
@@ -15082,6 +15243,9 @@
       <c r="Q3" s="4" t="n">
         <v>0.3165</v>
       </c>
+      <c r="R3" s="4" t="n">
+        <v>0.3165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15136,6 +15300,9 @@
       <c r="Q4" s="4" t="n">
         <v>0.6835</v>
       </c>
+      <c r="R4" s="4" t="n">
+        <v>0.6835</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15200,6 +15367,10 @@
         <f>SUM(Q3:Q4)</f>
         <v/>
       </c>
+      <c r="R5" s="5">
+        <f>SUM(R3:R4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15254,6 +15425,9 @@
       <c r="Q6" s="4" t="n">
         <v>0.0452</v>
       </c>
+      <c r="R6" s="4" t="n">
+        <v>0.0452</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15308,6 +15482,9 @@
       <c r="Q7" s="4" t="n">
         <v>0.0261</v>
       </c>
+      <c r="R7" s="4" t="n">
+        <v>0.0261</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15362,6 +15539,9 @@
       <c r="Q8" s="4" t="n">
         <v>0.0009</v>
       </c>
+      <c r="R8" s="4" t="n">
+        <v>0.0009</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15416,6 +15596,9 @@
       <c r="Q9" s="4" t="n">
         <v>0.0142</v>
       </c>
+      <c r="R9" s="4" t="n">
+        <v>0.0142</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15470,6 +15653,9 @@
       <c r="Q10" s="4" t="n">
         <v>0.2225</v>
       </c>
+      <c r="R10" s="4" t="n">
+        <v>0.2225</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -15524,6 +15710,9 @@
       <c r="Q11" s="4" t="n">
         <v>0.2101</v>
       </c>
+      <c r="R11" s="4" t="n">
+        <v>0.2101</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15578,6 +15767,9 @@
       <c r="Q12" s="4" t="n">
         <v>0.08310000000000001</v>
       </c>
+      <c r="R12" s="4" t="n">
+        <v>0.08310000000000001</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -15632,7 +15824,10 @@
       <c r="Q13" s="4" t="n">
         <v>0.33</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="R13" s="4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -15691,6 +15886,9 @@
       <c r="Q14" s="4" t="n">
         <v>0.001</v>
       </c>
+      <c r="R14" s="4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15745,6 +15943,9 @@
       <c r="Q15" s="4" t="n">
         <v>0.0624</v>
       </c>
+      <c r="R15" s="4" t="n">
+        <v>0.0624</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15796,6 +15997,9 @@
       <c r="Q16" s="4" t="n">
         <v>0.0013</v>
       </c>
+      <c r="R16" s="4" t="n">
+        <v>0.0013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15860,6 +16064,10 @@
         <f>SUM(Q6:Q16)</f>
         <v/>
       </c>
+      <c r="R17" s="5">
+        <f>SUM(R6:R16)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15914,6 +16122,9 @@
       <c r="Q18" s="4" t="n">
         <v>0.0276</v>
       </c>
+      <c r="R18" s="4" t="n">
+        <v>0.0276</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15968,6 +16179,9 @@
       <c r="Q19" s="4" t="n">
         <v>0.2141</v>
       </c>
+      <c r="R19" s="4" t="n">
+        <v>0.2157</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16022,6 +16236,9 @@
       <c r="Q20" s="4" t="n">
         <v>0.0175</v>
       </c>
+      <c r="R20" s="4" t="n">
+        <v>0.0175</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16073,7 +16290,10 @@
       <c r="Q21" s="4" t="n">
         <v>0.35</v>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="R21" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S21" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -16114,6 +16334,9 @@
       <c r="Q22" s="4" t="n">
         <v>0.0043</v>
       </c>
+      <c r="R22" s="4" t="n">
+        <v>0.0043</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -16144,6 +16367,9 @@
       <c r="Q23" s="4" t="n">
         <v>0.0086</v>
       </c>
+      <c r="R23" s="4" t="n">
+        <v>0.0167</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16168,6 +16394,9 @@
       <c r="Q24" s="4" t="n">
         <v>0.006</v>
       </c>
+      <c r="R24" s="4" t="n">
+        <v>0.006</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16232,6 +16461,10 @@
         <f>SUM(Q18:Q24)</f>
         <v/>
       </c>
+      <c r="R25" s="5">
+        <f>SUM(R18:R24)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -16286,6 +16519,9 @@
       <c r="Q26" s="4" t="n">
         <v>0.2462</v>
       </c>
+      <c r="R26" s="4" t="n">
+        <v>0.2462</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -16340,6 +16576,9 @@
       <c r="Q27" s="4" t="n">
         <v>0.08960000000000001</v>
       </c>
+      <c r="R27" s="4" t="n">
+        <v>0.08960000000000001</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -16394,7 +16633,10 @@
       <c r="Q28" s="4" t="n">
         <v>0.25</v>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="R28" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S28" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -16453,6 +16695,9 @@
       <c r="Q29" s="4" t="n">
         <v>0.04940000000000001</v>
       </c>
+      <c r="R29" s="4" t="n">
+        <v>0.04940000000000001</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16507,6 +16752,9 @@
       <c r="Q30" s="4" t="n">
         <v>0.0533</v>
       </c>
+      <c r="R30" s="4" t="n">
+        <v>0.0533</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -16561,6 +16809,9 @@
       <c r="Q31" s="4" t="n">
         <v>0.1124</v>
       </c>
+      <c r="R31" s="4" t="n">
+        <v>0.1124</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -16612,6 +16863,9 @@
       <c r="Q32" s="4" t="n">
         <v>0.1044</v>
       </c>
+      <c r="R32" s="4" t="n">
+        <v>0.1044</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16663,6 +16917,9 @@
       <c r="Q33" s="4" t="n">
         <v>0.0226</v>
       </c>
+      <c r="R33" s="4" t="n">
+        <v>0.0226</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -16714,6 +16971,9 @@
       <c r="Q34" s="4" t="n">
         <v>0.0369</v>
       </c>
+      <c r="R34" s="4" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -16762,6 +17022,9 @@
       <c r="Q35" s="4" t="n">
         <v>0.0014</v>
       </c>
+      <c r="R35" s="4" t="n">
+        <v>0.0014</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -16801,6 +17064,9 @@
       <c r="Q36" s="4" t="n">
         <v>0.0273</v>
       </c>
+      <c r="R36" s="4" t="n">
+        <v>0.0273</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -16831,6 +17097,9 @@
       <c r="Q37" s="4" t="n">
         <v>0.0027</v>
       </c>
+      <c r="R37" s="4" t="n">
+        <v>0.0027</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -16861,6 +17130,9 @@
       <c r="Q38" s="4" t="n">
         <v>0.0002</v>
       </c>
+      <c r="R38" s="4" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -16888,6 +17160,9 @@
       <c r="Q39" s="4" t="n">
         <v>0.0005999999999999999</v>
       </c>
+      <c r="R39" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16952,6 +17227,10 @@
         <f>SUM(Q26:Q39)</f>
         <v/>
       </c>
+      <c r="R40" s="5">
+        <f>SUM(R26:R39)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -17006,6 +17285,9 @@
       <c r="Q41" s="4" t="n">
         <v>0.2142</v>
       </c>
+      <c r="R41" s="4" t="n">
+        <v>0.2142</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -17060,6 +17342,9 @@
       <c r="Q42" s="4" t="n">
         <v>0.3459</v>
       </c>
+      <c r="R42" s="4" t="n">
+        <v>0.3459</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -17111,6 +17396,9 @@
       <c r="Q43" s="4" t="n">
         <v>0.0007000000000000001</v>
       </c>
+      <c r="R43" s="4" t="n">
+        <v>0.0007000000000000001</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -17150,6 +17438,9 @@
       <c r="Q44" s="4" t="n">
         <v>0.4389</v>
       </c>
+      <c r="R44" s="4" t="n">
+        <v>0.4389</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -17174,6 +17465,9 @@
       <c r="Q45" s="4" t="n">
         <v>0.0003</v>
       </c>
+      <c r="R45" s="4" t="n">
+        <v>0.0003</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -17238,6 +17532,10 @@
         <f>SUM(Q41:Q45)</f>
         <v/>
       </c>
+      <c r="R46" s="5">
+        <f>SUM(R41:R45)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -17292,6 +17590,9 @@
       <c r="Q47" s="4" t="n">
         <v>0.0025</v>
       </c>
+      <c r="R47" s="4" t="n">
+        <v>0.0025</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -17346,6 +17647,9 @@
       <c r="Q48" s="4" t="n">
         <v>0.4215</v>
       </c>
+      <c r="R48" s="4" t="n">
+        <v>0.4215</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -17400,6 +17704,9 @@
       <c r="Q49" s="4" t="n">
         <v>0.1712</v>
       </c>
+      <c r="R49" s="4" t="n">
+        <v>0.1712</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -17454,6 +17761,9 @@
       <c r="Q50" s="4" t="n">
         <v>0.016</v>
       </c>
+      <c r="R50" s="4" t="n">
+        <v>0.016</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -17508,6 +17818,9 @@
       <c r="Q51" s="4" t="n">
         <v>0.0133</v>
       </c>
+      <c r="R51" s="4" t="n">
+        <v>0.0133</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -17562,6 +17875,9 @@
       <c r="Q52" s="4" t="n">
         <v>0.0708</v>
       </c>
+      <c r="R52" s="4" t="n">
+        <v>0.0708</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -17613,6 +17929,9 @@
       <c r="Q53" s="4" t="n">
         <v>0.0072</v>
       </c>
+      <c r="R53" s="4" t="n">
+        <v>0.0095</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -17664,6 +17983,9 @@
       <c r="Q54" s="4" t="n">
         <v>0.2923</v>
       </c>
+      <c r="R54" s="4" t="n">
+        <v>0.2923</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -17712,6 +18034,9 @@
       <c r="Q55" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R55" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -17760,6 +18085,9 @@
       <c r="Q56" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R56" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -17808,6 +18136,9 @@
       <c r="Q57" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="R57" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -17856,6 +18187,9 @@
       <c r="Q58" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="R58" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -17904,6 +18238,9 @@
       <c r="Q59" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R59" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -17949,6 +18286,9 @@
       <c r="Q60" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R60" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -17994,6 +18334,9 @@
       <c r="Q61" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R61" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -18036,6 +18379,9 @@
       <c r="Q62" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R62" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -18075,6 +18421,9 @@
       <c r="Q63" s="4" t="n">
         <v>0.0001</v>
       </c>
+      <c r="R63" s="4" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -18139,6 +18488,10 @@
         <f>SUM(Q47:Q63)</f>
         <v/>
       </c>
+      <c r="R64" s="5">
+        <f>SUM(R47:R63)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -18193,6 +18546,9 @@
       <c r="Q65" s="4" t="n">
         <v>0.3348</v>
       </c>
+      <c r="R65" s="4" t="n">
+        <v>0.3361</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -18247,6 +18603,9 @@
       <c r="Q66" s="4" t="n">
         <v>0.0698</v>
       </c>
+      <c r="R66" s="4" t="n">
+        <v>0.0698</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -18301,6 +18660,9 @@
       <c r="Q67" s="4" t="n">
         <v>0.4926</v>
       </c>
+      <c r="R67" s="4" t="n">
+        <v>0.4926</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -18355,6 +18717,9 @@
       <c r="Q68" s="4" t="n">
         <v>0.0293</v>
       </c>
+      <c r="R68" s="4" t="n">
+        <v>0.0293</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -18403,6 +18768,9 @@
       <c r="Q69" s="4" t="n">
         <v>0.008500000000000001</v>
       </c>
+      <c r="R69" s="4" t="n">
+        <v>0.008500000000000001</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -18436,6 +18804,9 @@
       <c r="Q70" s="4" t="n">
         <v>0.0022</v>
       </c>
+      <c r="R70" s="4" t="n">
+        <v>0.0022</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -18500,6 +18871,10 @@
         <f>SUM(Q65:Q70)</f>
         <v/>
       </c>
+      <c r="R71" s="5">
+        <f>SUM(R65:R70)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -18554,6 +18929,9 @@
       <c r="Q72" s="4" t="n">
         <v>0.0021</v>
       </c>
+      <c r="R72" s="4" t="n">
+        <v>0.0021</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -18608,6 +18986,9 @@
       <c r="Q73" s="4" t="n">
         <v>0.0032</v>
       </c>
+      <c r="R73" s="4" t="n">
+        <v>0.0032</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -18662,6 +19043,9 @@
       <c r="Q74" s="4" t="n">
         <v>0.0204</v>
       </c>
+      <c r="R74" s="4" t="n">
+        <v>0.0204</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -18716,7 +19100,10 @@
       <c r="Q75" s="4" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="R75" t="inlineStr">
+      <c r="R75" s="4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="S75" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -18775,6 +19162,9 @@
       <c r="Q76" s="4" t="n">
         <v>0.0004</v>
       </c>
+      <c r="R76" s="4" t="n">
+        <v>0.0004</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -18829,6 +19219,9 @@
       <c r="Q77" s="4" t="n">
         <v>0.2828</v>
       </c>
+      <c r="R77" s="4" t="n">
+        <v>0.2828</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -18880,6 +19273,9 @@
       <c r="Q78" s="4" t="n">
         <v>0.0012</v>
       </c>
+      <c r="R78" s="4" t="n">
+        <v>0.0012</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -18928,6 +19324,9 @@
       <c r="Q79" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R79" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -18990,6 +19389,10 @@
       </c>
       <c r="Q80" s="5">
         <f>SUM(Q72:Q79)</f>
+        <v/>
+      </c>
+      <c r="R80" s="5">
+        <f>SUM(R72:R79)</f>
         <v/>
       </c>
     </row>
@@ -19004,7 +19407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19116,13 +19519,13 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>28</v>
+        <v>28.03</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>8.27</v>
+        <v>24.8</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>295.3571428571428</v>
+        <v>884.7663217980735</v>
       </c>
     </row>
     <row r="12">
@@ -19263,13 +19666,13 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>14409.51</v>
+        <v>16497.85</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>25027</v>
+        <v>28780.17</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1736.839073639562</v>
+        <v>1744.480038308022</v>
       </c>
     </row>
     <row r="19">
@@ -19347,13 +19750,13 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>971.6500000000001</v>
+        <v>1124.85</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>4207.960000000001</v>
+        <v>4886.18</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>4330.736376267175</v>
+        <v>4343.850291149932</v>
       </c>
     </row>
     <row r="23">
@@ -19452,13 +19855,13 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>70.61999999999999</v>
+        <v>79.92</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>176.62</v>
+        <v>195.69</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2500.991220617389</v>
+        <v>2448.573573573573</v>
       </c>
     </row>
     <row r="28">
@@ -19515,13 +19918,13 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>9083.459999999999</v>
+        <v>10517.34999999999</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>20469.96</v>
+        <v>23896.71000000001</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>2253.542152439709</v>
+        <v>2272.122730535736</v>
       </c>
     </row>
     <row r="31">
@@ -19536,13 +19939,13 @@
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>36.85999999999999</v>
+        <v>37.89999999999999</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>84.98</v>
+        <v>86.98</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>2305.480195333696</v>
+        <v>2294.986807387863</v>
       </c>
     </row>
     <row r="32">
@@ -19620,13 +20023,13 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>424.12</v>
+        <v>492.18</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>761.33</v>
+        <v>817.4100000000001</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>1795.081580684712</v>
+        <v>1660.794831159332</v>
       </c>
     </row>
     <row r="36">
@@ -19704,13 +20107,13 @@
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>11411.46</v>
+        <v>12738.41</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>21267.10999999999</v>
+        <v>23782.68</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1863.662493668645</v>
+        <v>1867.005379792298</v>
       </c>
     </row>
     <row r="40">
@@ -19725,13 +20128,13 @@
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>6722.290000000001</v>
+        <v>7213.89</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>7449.77</v>
+        <v>8054.110000000001</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>1108.219074154789</v>
+        <v>1116.472527304963</v>
       </c>
     </row>
     <row r="41">
@@ -19767,13 +20170,13 @@
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>1795.37</v>
+        <v>1868.6</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>2421.72</v>
+        <v>2475.41</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>1348.869592340298</v>
+        <v>1324.740447393771</v>
       </c>
     </row>
     <row r="43">
@@ -19809,13 +20212,13 @@
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>4841.26</v>
+        <v>4921.71</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>9501.809999999999</v>
+        <v>9661.15</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1962.672940515486</v>
+        <v>1962.966123562745</v>
       </c>
     </row>
     <row r="45">
@@ -19893,13 +20296,13 @@
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>17416.15</v>
+        <v>17430.11</v>
       </c>
       <c r="D48" s="6" t="n">
-        <v>28775.74</v>
+        <v>28817.23</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>1652.244612041122</v>
+        <v>1653.301671647512</v>
       </c>
     </row>
     <row r="49">
@@ -19910,17 +20313,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>663.12</v>
+        <v>84.97</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1537.45</v>
+        <v>96.47</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>2318.509470382435</v>
+        <v>1135.341885371308</v>
       </c>
     </row>
     <row r="50">
@@ -19931,17 +20334,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>85.22</v>
+        <v>829.95</v>
       </c>
       <c r="D50" s="6" t="n">
-        <v>144.14</v>
+        <v>1926.96</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>1691.386998357193</v>
+        <v>2321.77842038677</v>
       </c>
     </row>
     <row r="51">
@@ -19952,17 +20355,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>488.37</v>
+        <v>85.22</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>940.9100000000001</v>
+        <v>144.14</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>1926.633495095931</v>
+        <v>1691.386998357193</v>
       </c>
     </row>
     <row r="52">
@@ -19973,17 +20376,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>4562.59</v>
+        <v>488.37</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>5650.14</v>
+        <v>940.9100000000001</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>1238.362421344017</v>
+        <v>1926.633495095931</v>
       </c>
     </row>
     <row r="53">
@@ -19994,17 +20397,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>5.02</v>
+        <v>4689.37</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>24.36</v>
+        <v>5821.76</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>4852.589641434263</v>
+        <v>1241.480198832679</v>
       </c>
     </row>
     <row r="54">
@@ -20015,17 +20418,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>455.09</v>
+        <v>5.02</v>
       </c>
       <c r="D54" s="6" t="n">
-        <v>644.63</v>
+        <v>24.36</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>1416.489046122745</v>
+        <v>4852.589641434263</v>
       </c>
     </row>
     <row r="55">
@@ -20036,17 +20439,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>0.01</v>
+        <v>455.09</v>
       </c>
       <c r="D55" s="6" t="n">
-        <v>0.03</v>
+        <v>644.63</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>3000</v>
+        <v>1416.489046122745</v>
       </c>
     </row>
     <row r="56">
@@ -20057,17 +20460,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="D56" s="6" t="n">
-        <v>0.25</v>
+        <v>0.03</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>2083.333333333333</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="57">
@@ -20078,17 +20481,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>7295.74</v>
+        <v>0.12</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>11154.6</v>
+        <v>0.25</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>1528.91961610474</v>
+        <v>2083.333333333333</v>
       </c>
     </row>
     <row r="58">
@@ -20099,17 +20502,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>542.15</v>
+        <v>12664.74</v>
       </c>
       <c r="D58" s="6" t="n">
-        <v>737.62</v>
+        <v>17203.03</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>1360.545974361339</v>
+        <v>1358.340558116471</v>
       </c>
     </row>
     <row r="59">
@@ -20120,17 +20523,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>3687.78</v>
+        <v>542.15</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>4387.33</v>
+        <v>737.62</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>1189.694070687514</v>
+        <v>1360.545974361339</v>
       </c>
     </row>
     <row r="60">
@@ -20141,17 +20544,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C60" s="6" t="n">
-        <v>0.33</v>
+        <v>3687.78</v>
       </c>
       <c r="D60" s="6" t="n">
-        <v>1.37</v>
+        <v>4387.33</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>4151.515151515151</v>
+        <v>1189.694070687514</v>
       </c>
     </row>
     <row r="61">
@@ -20162,17 +20565,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>15.63</v>
+        <v>0.33</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>45.93</v>
+        <v>1.37</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>2938.579654510556</v>
+        <v>4151.515151515151</v>
       </c>
     </row>
     <row r="62">
@@ -20183,17 +20586,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C62" s="6" t="n">
-        <v>35556.35999999999</v>
+        <v>15.63</v>
       </c>
       <c r="D62" s="6" t="n">
-        <v>75316.79000000001</v>
+        <v>45.93</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>2118.236793642545</v>
+        <v>2938.579654510556</v>
       </c>
     </row>
     <row r="63">
@@ -20204,38 +20607,38 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C63" s="6" t="n">
-        <v>1988.28</v>
+        <v>39172.45</v>
       </c>
       <c r="D63" s="6" t="n">
-        <v>2548.99</v>
+        <v>83093.71000000005</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>1282.007564326956</v>
+        <v>2121.228312244959</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Rebar</t>
+          <t>Coated Steel Sheet</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="C64" s="6" t="n">
-        <v>133.1</v>
+        <v>1988.28</v>
       </c>
       <c r="D64" s="6" t="n">
-        <v>169.14</v>
+        <v>2548.99</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>1270.773854244928</v>
+        <v>1282.007564326956</v>
       </c>
     </row>
     <row r="65">
@@ -20246,17 +20649,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C65" s="6" t="n">
-        <v>19.72</v>
+        <v>133.1</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>39.63</v>
+        <v>169.14</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>2009.634888438134</v>
+        <v>1270.773854244928</v>
       </c>
     </row>
     <row r="66">
@@ -20267,17 +20670,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>7.31</v>
+        <v>19.72</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>19.98</v>
+        <v>39.63</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>2733.242134062928</v>
+        <v>2009.634888438134</v>
       </c>
     </row>
     <row r="67">
@@ -20288,17 +20691,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>2066.03</v>
+        <v>7.31</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>1573.68</v>
+        <v>19.98</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>761.6927150138189</v>
+        <v>2733.242134062928</v>
       </c>
     </row>
     <row r="68">
@@ -20309,17 +20712,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>9921.959999999999</v>
+        <v>2066.03</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>7484.200000000001</v>
+        <v>1573.68</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>754.3066087748794</v>
+        <v>761.6927150138189</v>
       </c>
     </row>
     <row r="69">
@@ -20330,17 +20733,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>9048.489999999998</v>
+        <v>9921.959999999999</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>12398.53</v>
+        <v>7484.200000000001</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1370.231939251743</v>
+        <v>754.3066087748794</v>
       </c>
     </row>
     <row r="70">
@@ -20351,17 +20754,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>49.88</v>
+        <v>9299.099999999999</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>80.97</v>
+        <v>12734.46</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>1623.295910184443</v>
+        <v>1369.42929960964</v>
       </c>
     </row>
     <row r="71">
@@ -20372,38 +20775,38 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>504.5500000000001</v>
+        <v>99.76000000000001</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>739.8299999999999</v>
+        <v>155.63</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>1466.316519670994</v>
+        <v>1560.04410585405</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Hot-Rolled Bar</t>
+          <t>Rebar</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>166.21</v>
+        <v>605.9400000000001</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>362.5</v>
+        <v>874.8</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>2180.975873894471</v>
+        <v>1443.707297752253</v>
       </c>
     </row>
     <row r="73">
@@ -20414,17 +20817,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>28.89</v>
+        <v>173.57</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>51.74</v>
+        <v>378.35</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>1790.931118033922</v>
+        <v>2179.812179524111</v>
       </c>
     </row>
     <row r="74">
@@ -20435,17 +20838,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C74" s="6" t="n">
-        <v>645.63</v>
+        <v>200.14</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>1079.21</v>
+        <v>266.08</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>1671.561110852965</v>
+        <v>1329.469371439992</v>
       </c>
     </row>
     <row r="75">
@@ -20456,17 +20859,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>0.01</v>
+        <v>645.63</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>0.01</v>
+        <v>1079.21</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1000</v>
+        <v>1671.561110852965</v>
       </c>
     </row>
     <row r="76">
@@ -20477,17 +20880,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C76" s="6" t="n">
-        <v>680.04</v>
+        <v>0.01</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>1020.66</v>
+        <v>0.01</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>1500.882301041115</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="77">
@@ -20498,17 +20901,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>63.19</v>
+        <v>3.95</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>133.25</v>
+        <v>16.83</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>2108.719734135148</v>
+        <v>4260.759493670886</v>
       </c>
     </row>
     <row r="78">
@@ -20519,17 +20922,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>2231.47</v>
+        <v>880</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>2253.41</v>
+        <v>1374.45</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>1009.832083783336</v>
+        <v>1561.875</v>
       </c>
     </row>
     <row r="79">
@@ -20540,17 +20943,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C79" s="6" t="n">
-        <v>321.41</v>
+        <v>63.19</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>335.59</v>
+        <v>133.25</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>1044.118104601599</v>
+        <v>2108.719734135148</v>
       </c>
     </row>
     <row r="80">
@@ -20561,59 +20964,59 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>2987</v>
+        <v>2398.91</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>6399.969999999999</v>
+        <v>2434.17</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>2142.607967860729</v>
+        <v>1014.698342163733</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C81" s="6" t="n">
-        <v>72.08</v>
+        <v>321.41</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>104.06</v>
+        <v>335.59</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>1443.673695893452</v>
+        <v>1044.118104601599</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Wire Rod</t>
+          <t>Hot-Rolled Bar</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C82" s="6" t="n">
-        <v>385.82</v>
+        <v>3363.5</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>496.14</v>
+        <v>7237.199999999998</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>1285.936447047846</v>
+        <v>2151.687230563401</v>
       </c>
     </row>
     <row r="83">
@@ -20624,17 +21027,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C83" s="6" t="n">
-        <v>5714.400000000001</v>
+        <v>72.08</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>7504.52</v>
+        <v>104.06</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>1313.264734705306</v>
+        <v>1443.673695893452</v>
       </c>
     </row>
     <row r="84">
@@ -20645,17 +21048,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>1.83</v>
+        <v>745.3499999999999</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>5.66</v>
+        <v>1002.02</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>3092.896174863388</v>
+        <v>1344.361709264104</v>
       </c>
     </row>
     <row r="85">
@@ -20666,17 +21069,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>88.08000000000001</v>
+        <v>6480.490000000001</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>147.89</v>
+        <v>8480.98</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>1679.041780199818</v>
+        <v>1308.694249971838</v>
       </c>
     </row>
     <row r="86">
@@ -20687,17 +21090,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>2679.14</v>
+        <v>1.83</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>2208.72</v>
+        <v>5.66</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>824.4138044297797</v>
+        <v>3092.896174863388</v>
       </c>
     </row>
     <row r="87">
@@ -20708,17 +21111,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>95.56999999999999</v>
+        <v>88.08000000000001</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>256.16</v>
+        <v>147.89</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>2680.339018520457</v>
+        <v>1679.041780199818</v>
       </c>
     </row>
     <row r="88">
@@ -20729,17 +21132,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>193.25</v>
+        <v>2679.14</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>263.71</v>
+        <v>2208.72</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>1364.605433376456</v>
+        <v>824.4138044297797</v>
       </c>
     </row>
     <row r="89">
@@ -20750,17 +21153,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C89" s="6" t="n">
-        <v>93.3</v>
+        <v>95.56999999999999</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>138.03</v>
+        <v>256.16</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>1479.421221864952</v>
+        <v>2680.339018520457</v>
       </c>
     </row>
     <row r="90">
@@ -20771,17 +21174,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>297.7</v>
+        <v>193.25</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>389.33</v>
+        <v>263.71</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>1307.793080282163</v>
+        <v>1364.605433376456</v>
       </c>
     </row>
     <row r="91">
@@ -20792,59 +21195,59 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>7342.349999999999</v>
+        <v>93.3</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>11178.65</v>
+        <v>138.03</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>1522.489393722719</v>
+        <v>1479.421221864952</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>2420.79</v>
+        <v>297.7</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>2123.93</v>
+        <v>389.33</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>877.3706104205654</v>
+        <v>1307.793080282163</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Structural Steel</t>
+          <t>Wire Rod</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>1.15</v>
+        <v>8103.02</v>
       </c>
       <c r="D93" s="6" t="n">
-        <v>2.14</v>
+        <v>12269.07</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>1860.869565217391</v>
+        <v>1514.135470478908</v>
       </c>
     </row>
     <row r="94">
@@ -20855,17 +21258,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C94" s="6" t="n">
-        <v>388.01</v>
+        <v>2420.79</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>1254.6</v>
+        <v>2123.93</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>3233.421819025283</v>
+        <v>877.3706104205654</v>
       </c>
     </row>
     <row r="95">
@@ -20876,17 +21279,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C95" s="6" t="n">
-        <v>55.54</v>
+        <v>1.15</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>81.45</v>
+        <v>2.14</v>
       </c>
       <c r="E95" s="6" t="n">
-        <v>1466.510622974433</v>
+        <v>1860.869565217391</v>
       </c>
     </row>
     <row r="96">
@@ -20897,17 +21300,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C96" s="6" t="n">
-        <v>17.16</v>
+        <v>388.11</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>80.98999999999999</v>
+        <v>1255.37</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>4719.69696969697</v>
+        <v>3234.572672695885</v>
       </c>
     </row>
     <row r="97">
@@ -20918,17 +21321,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C97" s="6" t="n">
-        <v>824.29</v>
+        <v>55.54</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>926.6900000000001</v>
+        <v>81.45</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>1124.228123597278</v>
+        <v>1466.510622974433</v>
       </c>
     </row>
     <row r="98">
@@ -20939,17 +21342,17 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Korea, Republic of</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C98" s="6" t="n">
-        <v>32984.2</v>
+        <v>18</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>34707.86</v>
+        <v>85.08</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1052.257141297955</v>
+        <v>4726.666666666668</v>
       </c>
     </row>
     <row r="99">
@@ -20960,17 +21363,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C99" s="6" t="n">
-        <v>10982.17</v>
+        <v>824.29</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>17973.24</v>
+        <v>926.6900000000001</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>1636.583662427371</v>
+        <v>1124.228123597278</v>
       </c>
     </row>
     <row r="100">
@@ -20981,17 +21384,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Korea, Republic of</t>
         </is>
       </c>
       <c r="C100" s="6" t="n">
-        <v>8497.539999999999</v>
+        <v>32984.2</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>13331.46</v>
+        <v>34707.86</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1568.861105684704</v>
+        <v>1052.257141297955</v>
       </c>
     </row>
     <row r="101">
@@ -21002,17 +21405,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C101" s="6" t="n">
-        <v>2</v>
+        <v>10982.17</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>3.57</v>
+        <v>17973.24</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>1785</v>
+        <v>1636.583662427371</v>
       </c>
     </row>
     <row r="102">
@@ -21023,17 +21426,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="C102" s="6" t="n">
-        <v>12031.83</v>
+        <v>9981.849999999999</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>14194.2</v>
+        <v>16002.43</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>1179.720790602925</v>
+        <v>1603.152722190777</v>
       </c>
     </row>
     <row r="103">
@@ -21044,17 +21447,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C103" s="6" t="n">
-        <v>0.05</v>
+        <v>2</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>0.24</v>
+        <v>3.57</v>
       </c>
       <c r="E103" s="6" t="n">
-        <v>4800</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="104">
@@ -21065,17 +21468,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C104" s="6" t="n">
-        <v>653.25</v>
+        <v>12058.65</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>636.14</v>
+        <v>14333.39</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>973.80788365863</v>
+        <v>1188.639690180908</v>
       </c>
     </row>
     <row r="105">
@@ -21086,17 +21489,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C105" s="6" t="n">
-        <v>20116.69</v>
+        <v>0.05</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>18313.92</v>
+        <v>0.24</v>
       </c>
       <c r="E105" s="6" t="n">
-        <v>910.3843624373593</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="106">
@@ -21107,17 +21510,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>637.12</v>
+        <v>676.89</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>972.5999999999999</v>
+        <v>659.0599999999999</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>1526.557006529382</v>
+        <v>973.6589401527575</v>
       </c>
     </row>
     <row r="107">
@@ -21128,17 +21531,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="C107" s="6" t="n">
-        <v>328.9</v>
+        <v>20116.69</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>438.0000000000001</v>
+        <v>18313.92</v>
       </c>
       <c r="E107" s="6" t="n">
-        <v>1331.711766494376</v>
+        <v>910.3843624373593</v>
       </c>
     </row>
     <row r="108">
@@ -21149,17 +21552,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="C108" s="6" t="n">
-        <v>8429.839999999997</v>
+        <v>637.1800000000001</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>21945.02</v>
+        <v>972.8299999999999</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>2603.254628794853</v>
+        <v>1526.774223924165</v>
       </c>
     </row>
     <row r="109">
@@ -21170,16 +21573,58 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>329.01</v>
+      </c>
+      <c r="D109" s="6" t="n">
+        <v>438.59</v>
+      </c>
+      <c r="E109" s="6" t="n">
+        <v>1333.059785416857</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n">
+        <v>9509.679999999998</v>
+      </c>
+      <c r="D110" s="6" t="n">
+        <v>24837.41000000001</v>
+      </c>
+      <c r="E110" s="6" t="n">
+        <v>2611.80292081332</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Structural Steel</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="C109" s="6" t="n">
+      <c r="C111" s="6" t="n">
         <v>690.49</v>
       </c>
-      <c r="D109" s="6" t="n">
+      <c r="D111" s="6" t="n">
         <v>579.4100000000001</v>
       </c>
-      <c r="E109" s="6" t="n">
+      <c r="E111" s="6" t="n">
         <v>839.1287346666861</v>
       </c>
     </row>

</xml_diff>